<commit_message>
Kapitel 3 überarbeitet. Noch nicht verländert
</commit_message>
<xml_diff>
--- a/notes/Zeitplan.xlsx
+++ b/notes/Zeitplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://altengroup-my.sharepoint.com/personal/isabel_norpoth_alten-worldgrid_com/Documents/Dokumente/Masterarbeit/notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="11_AD4DB114E441178AC67DF4641692EAA0683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D1FF0A-A650-4DAB-88DC-B1F86C60C8BC}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="11_AD4DB114E441178AC67DF4641692EAA0683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6913F5E8-D0DC-4008-9614-C7AA5F2CBA0E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -196,7 +196,7 @@
   </si>
   <si>
     <t>14.09.
-- iojfijsoid</t>
+- Format angepasst</t>
   </si>
 </sst>
 </file>
@@ -280,6 +280,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -565,7 +569,15 @@
   <dimension ref="B2:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="10" width="9.109375" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" customWidth="1"/>
     <col min="11" max="11" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -595,7 +607,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Zeilenumbruch bei code funktioniert noch nicht, sonst format passt
</commit_message>
<xml_diff>
--- a/notes/Zeitplan.xlsx
+++ b/notes/Zeitplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://altengroup-my.sharepoint.com/personal/isabel_norpoth_alten-worldgrid_com/Documents/Dokumente/Masterarbeit/notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="11_AD4DB114E441178AC67DF4641692EAA0683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6913F5E8-D0DC-4008-9614-C7AA5F2CBA0E}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="11_AD4DB114E441178AC67DF4641692EAA0683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81E139D9-DD7B-4C82-A2DE-B45832C4731B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38490" yWindow="-13910" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -51,18 +51,6 @@
     <t>KW</t>
   </si>
   <si>
-    <t>15.09.</t>
-  </si>
-  <si>
-    <t>16.09.</t>
-  </si>
-  <si>
-    <t>17.09.</t>
-  </si>
-  <si>
-    <t>18.09.</t>
-  </si>
-  <si>
     <t>19.09.</t>
   </si>
   <si>
@@ -197,6 +185,25 @@
   <si>
     <t>14.09.
 - Format angepasst</t>
+  </si>
+  <si>
+    <t>17.09.
+- Nichts</t>
+  </si>
+  <si>
+    <t>16.09.
+- Format angepasst
+- Qellen Kapitel 3 hinzugefügt</t>
+  </si>
+  <si>
+    <t>15.09.
+- Kapitel 3 überarbeitet</t>
+  </si>
+  <si>
+    <t>18.09.
+- Abkürzungsverzeichnis repariert
+- letztes Kommentar aus Kapitel 3 angepasst
+- Beginn Quellen zu 4. hinzuzufügen</t>
   </si>
 </sst>
 </file>
@@ -232,42 +239,54 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+  <dxfs count="10">
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -287,17 +306,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21100D2E-E902-4139-BEFD-4242AD9F1908}" name="Tabelle1" displayName="Tabelle1" ref="B2:I9" totalsRowShown="0">
-  <autoFilter ref="B2:I9" xr:uid="{21100D2E-E902-4139-BEFD-4242AD9F1908}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{21100D2E-E902-4139-BEFD-4242AD9F1908}" name="Tabelle1" displayName="Tabelle1" ref="B3:I10" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="B3:I10" xr:uid="{21100D2E-E902-4139-BEFD-4242AD9F1908}"/>
   <tableColumns count="8">
-    <tableColumn id="11" xr3:uid="{05CB0716-A1A2-46A0-9EEC-0606C1EFE3B1}" name="KW"/>
-    <tableColumn id="1" xr3:uid="{654640F4-9C35-4F2C-8DE9-F9B6654E20FD}" name="Montag" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7BE82199-C101-4AD5-8DA5-BE3C54A30A9F}" name="Dienstag" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{0B6803C4-59E6-4A83-9ED1-3A6BF5E00E7A}" name="Mittwoch" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{9EEC4867-53E8-4FF7-B101-D3A39FE605B2}" name="Donnerstag" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{5D8E4842-0643-440A-9AAD-0442AB5841DA}" name="Freitag" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{45542995-F8E0-4890-BC59-E36DA995D04B}" name="Samstag" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{772ECBD7-8078-4192-93F3-F78DDE52A9C8}" name="Sonntag" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{05CB0716-A1A2-46A0-9EEC-0606C1EFE3B1}" name="KW" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{654640F4-9C35-4F2C-8DE9-F9B6654E20FD}" name="Montag" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{7BE82199-C101-4AD5-8DA5-BE3C54A30A9F}" name="Dienstag" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{0B6803C4-59E6-4A83-9ED1-3A6BF5E00E7A}" name="Mittwoch" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{9EEC4867-53E8-4FF7-B101-D3A39FE605B2}" name="Donnerstag" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{5D8E4842-0643-440A-9AAD-0442AB5841DA}" name="Freitag" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{45542995-F8E0-4890-BC59-E36DA995D04B}" name="Samstag" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{772ECBD7-8078-4192-93F3-F78DDE52A9C8}" name="Sonntag" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -566,227 +585,237 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:I9"/>
+  <dimension ref="A2:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.109375" customWidth="1"/>
     <col min="11" max="11" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B3" s="1">
+    <row r="4" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2">
         <v>38</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3" t="s">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2">
+        <v>39</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="G5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="1">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2">
+        <v>40</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2">
+        <v>41</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2">
+        <v>42</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>20</v>
+      <c r="I8" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B5" s="1">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2">
+        <v>43</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="D9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="3" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="2">
+        <v>44</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B6" s="1">
-        <v>41</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="1">
-        <v>42</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B8" s="1">
-        <v>43</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B9" s="1">
-        <v>44</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>